<commit_message>
Restored local changes to PositionTransduserRun1 and TODOKladd
</commit_message>
<xml_diff>
--- a/data/CylinderTransduser/PositionTransduserRun1.xlsx
+++ b/data/CylinderTransduser/PositionTransduserRun1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sujro\Documents\GitHub\Bachelor\data\CylinderTransduser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC772AA5-7489-4B51-BB58-EFD59D103F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3E6877-21E3-4224-ABA5-A8198930C432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{AD92D090-37B1-4D85-9043-B221BBD43E04}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
   <si>
     <t>Fysisk måling [m]</t>
   </si>
@@ -72,12 +72,6 @@
   </si>
   <si>
     <t>spool_down</t>
-  </si>
-  <si>
-    <t>delta</t>
-  </si>
-  <si>
-    <t>skaleringsfeil her må fikse</t>
   </si>
 </sst>
 </file>
@@ -168,15 +162,15 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -654,6 +648,71 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="log"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="6"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0.13766956897552923"/>
+                  <c:y val="-0.59456863239978419"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="nb-NO"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>cylinder!$B$18:$B$28</c:f>
@@ -706,31 +765,31 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-9.9999999999999395E-4</c:v>
+                  <c:v>9.9999999999999395E-4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-1.0000000000000009E-3</c:v>
+                  <c:v>1.0000000000000009E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-9.000000000000008E-3</c:v>
+                  <c:v>9.000000000000008E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-1.2999999999999984E-2</c:v>
+                  <c:v>1.2999999999999984E-2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-1.7000000000000015E-2</c:v>
+                  <c:v>1.7000000000000015E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-1.8500000000000016E-2</c:v>
+                  <c:v>1.8500000000000016E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-1.9000000000000017E-2</c:v>
+                  <c:v>1.9000000000000017E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-1.4999999999999958E-2</c:v>
+                  <c:v>1.4999999999999958E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-1.0000000000000009E-2</c:v>
+                  <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -932,6 +991,423 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="nb-NO"/>
+              <a:t>uReal</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="nb-NO" baseline="0"/>
+              <a:t> vs uSignal, up</a:t>
+            </a:r>
+            <a:endParaRPr lang="nb-NO"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="nb-NO"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>cylinder!$B$40:$B$55</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="16"/>
+                <c:pt idx="0">
+                  <c:v>0.25</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.35</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.45</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.55000000000000004</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.65</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.7</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.75</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.8</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.85</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.9</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.95</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>cylinder!$C$40:$C$55</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="16"/>
+                <c:pt idx="0">
+                  <c:v>0.246124941286989</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.30366369187411901</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.35979333020197202</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.413574448097698</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.470173790511977</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.52489431658055397</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.58243306716768395</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.63856270549553695</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.69751056834194403</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.75082198215124396</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.80742132456552296</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.86261155472052597</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.91498356035697503</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.973461719116956</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-40B4-43EB-8ADC-FB51E39106BD}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1219934543"/>
+        <c:axId val="895625519"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1219934543"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="nb-NO"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="895625519"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="895625519"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="nb-NO"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1219934543"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="nb-NO"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1012,6 +1488,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -1529,6 +2045,522 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2113,6 +3145,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>388143</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>147637</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>123824</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{872554EF-334C-9439-FD82-FB446033CCEC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2449,11 +3517,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.5">
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
     </row>
     <row r="2" spans="1:8" ht="15.4" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" s="6" t="s">
@@ -2622,11 +3690,11 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="15" x14ac:dyDescent="0.5">
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
     </row>
     <row r="17" spans="2:15" ht="15.4" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B17" s="6" t="s">
@@ -2647,7 +3715,7 @@
         <v>0</v>
       </c>
       <c r="D18" s="5">
-        <f t="shared" ref="D18:D28" si="1">B18-C18</f>
+        <f>C18-B18</f>
         <v>0</v>
       </c>
     </row>
@@ -2659,8 +3727,8 @@
         <v>5.0999999999999997E-2</v>
       </c>
       <c r="D19" s="5">
-        <f t="shared" si="1"/>
-        <v>-9.9999999999999395E-4</v>
+        <f t="shared" ref="D19:D28" si="1">C19-B19</f>
+        <v>9.9999999999999395E-4</v>
       </c>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.45">
@@ -2672,7 +3740,7 @@
       </c>
       <c r="D20" s="5">
         <f t="shared" si="1"/>
-        <v>-1.0000000000000009E-3</v>
+        <v>1.0000000000000009E-3</v>
       </c>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.45">
@@ -2684,7 +3752,7 @@
       </c>
       <c r="D21" s="5">
         <f t="shared" si="1"/>
-        <v>-9.000000000000008E-3</v>
+        <v>9.000000000000008E-3</v>
       </c>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.45">
@@ -2696,7 +3764,7 @@
       </c>
       <c r="D22" s="5">
         <f t="shared" si="1"/>
-        <v>-1.2999999999999984E-2</v>
+        <v>1.2999999999999984E-2</v>
       </c>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.45">
@@ -2708,7 +3776,7 @@
       </c>
       <c r="D23" s="5">
         <f t="shared" si="1"/>
-        <v>-1.7000000000000015E-2</v>
+        <v>1.7000000000000015E-2</v>
       </c>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.45">
@@ -2720,7 +3788,7 @@
       </c>
       <c r="D24" s="5">
         <f t="shared" si="1"/>
-        <v>-1.8500000000000016E-2</v>
+        <v>1.8500000000000016E-2</v>
       </c>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.45">
@@ -2732,7 +3800,7 @@
       </c>
       <c r="D25" s="5">
         <f t="shared" si="1"/>
-        <v>-1.9000000000000017E-2</v>
+        <v>1.9000000000000017E-2</v>
       </c>
       <c r="O25" t="s">
         <v>7</v>
@@ -2747,7 +3815,7 @@
       </c>
       <c r="D26" s="5">
         <f t="shared" si="1"/>
-        <v>-1.4999999999999958E-2</v>
+        <v>1.4999999999999958E-2</v>
       </c>
     </row>
     <row r="27" spans="2:15" x14ac:dyDescent="0.45">
@@ -2759,7 +3827,7 @@
       </c>
       <c r="D27" s="5">
         <f t="shared" si="1"/>
-        <v>-1.0000000000000009E-2</v>
+        <v>1.0000000000000009E-2</v>
       </c>
     </row>
     <row r="28" spans="2:15" x14ac:dyDescent="0.45">
@@ -2774,15 +3842,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="15" x14ac:dyDescent="0.5">
-      <c r="B38" s="7" t="s">
+    <row r="38" spans="2:5" ht="15" x14ac:dyDescent="0.5">
+      <c r="B38" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="7"/>
-    </row>
-    <row r="39" spans="2:7" ht="15.4" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+    </row>
+    <row r="39" spans="2:5" ht="15.4" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B39" s="6" t="s">
         <v>9</v>
       </c>
@@ -2792,152 +3860,147 @@
       <c r="D39" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E39" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="E39" s="6"/>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B40" s="5">
         <v>0.25</v>
       </c>
-      <c r="C40" s="10">
-        <v>0.51</v>
+      <c r="C40" s="8">
+        <v>0.246124941286989</v>
       </c>
       <c r="D40" s="5"/>
-      <c r="E40" s="9"/>
-    </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="E40" s="7"/>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B41" s="5">
         <v>0.3</v>
       </c>
-      <c r="C41" s="10">
-        <v>0.61834733893557403</v>
+      <c r="C41" s="8">
+        <v>0.30366369187411901</v>
       </c>
       <c r="D41" s="5"/>
-      <c r="E41" s="9"/>
-    </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="E41" s="7"/>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B42" s="5">
         <v>0.35</v>
       </c>
-      <c r="C42" s="10">
-        <v>0.72665732959850604</v>
+      <c r="C42" s="8">
+        <v>0.35979333020197202</v>
       </c>
       <c r="D42" s="5"/>
-      <c r="E42" s="9"/>
-    </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="E42" s="7"/>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B43" s="5">
         <v>0.4</v>
       </c>
-      <c r="C43" s="10">
-        <v>0.83099906629318399</v>
+      <c r="C43" s="8">
+        <v>0.413574448097698</v>
       </c>
       <c r="D43" s="5"/>
-      <c r="E43" s="9"/>
-    </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="E43" s="7"/>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B44" s="5">
         <v>0.45</v>
       </c>
-      <c r="C44" s="10">
-        <v>0.93580765639589103</v>
+      <c r="C44" s="8">
+        <v>0.470173790511977</v>
       </c>
       <c r="D44" s="5"/>
-      <c r="E44" s="9"/>
-    </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="E44" s="7"/>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B45" s="5">
         <v>0.5</v>
       </c>
       <c r="C45" s="5">
-        <v>1</v>
+        <v>0.52489431658055397</v>
       </c>
       <c r="D45" s="5"/>
-      <c r="E45" s="9"/>
-    </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="E45" s="7"/>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B46" s="5">
         <v>0.55000000000000004</v>
       </c>
       <c r="C46" s="5">
-        <v>1</v>
+        <v>0.58243306716768395</v>
       </c>
       <c r="D46" s="5"/>
-      <c r="E46" s="9"/>
-    </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="E46" s="7"/>
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B47" s="5">
         <v>0.6</v>
       </c>
       <c r="C47" s="5">
-        <v>1</v>
+        <v>0.63856270549553695</v>
       </c>
       <c r="D47" s="5"/>
-      <c r="E47" s="9"/>
-      <c r="G47" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="E47" s="7"/>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B48" s="5">
         <v>0.65</v>
       </c>
       <c r="C48" s="5">
-        <v>1</v>
+        <v>0.69751056834194403</v>
       </c>
       <c r="D48" s="5"/>
-      <c r="E48" s="9"/>
+      <c r="E48" s="7"/>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B49" s="5">
         <v>0.7</v>
       </c>
       <c r="C49" s="5">
-        <v>1</v>
+        <v>0.75082198215124396</v>
       </c>
       <c r="D49" s="5"/>
-      <c r="E49" s="9"/>
+      <c r="E49" s="7"/>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B50" s="5">
         <v>0.75</v>
       </c>
       <c r="C50" s="5">
-        <v>1</v>
+        <v>0.80742132456552296</v>
       </c>
       <c r="D50" s="5"/>
-      <c r="E50" s="9"/>
+      <c r="E50" s="7"/>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B51" s="5">
         <v>0.8</v>
       </c>
       <c r="C51" s="5">
-        <v>1</v>
-      </c>
-      <c r="D51" s="9"/>
-      <c r="E51" s="9"/>
+        <v>0.86261155472052597</v>
+      </c>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B52" s="5">
         <v>0.85</v>
       </c>
       <c r="C52" s="5">
-        <v>1</v>
-      </c>
-      <c r="D52" s="9"/>
-      <c r="E52" s="9"/>
+        <v>0.91498356035697503</v>
+      </c>
+      <c r="D52" s="7"/>
+      <c r="E52" s="7"/>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B53" s="5">
         <v>0.9</v>
       </c>
       <c r="C53" s="5">
-        <v>1</v>
-      </c>
-      <c r="D53" s="9"/>
-      <c r="E53" s="9"/>
+        <v>0.973461719116956</v>
+      </c>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B54" s="5">
@@ -2946,8 +4009,8 @@
       <c r="C54" s="5">
         <v>1</v>
       </c>
-      <c r="D54" s="9"/>
-      <c r="E54" s="9"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B55" s="5">
@@ -2956,8 +4019,8 @@
       <c r="C55" s="5">
         <v>1</v>
       </c>
-      <c r="D55" s="9"/>
-      <c r="E55" s="9"/>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>